<commit_message>
Add se_fallback manifest field for deriving missing SE from n
Opt-in, same hard-error-without-reason pattern as placebo_clamp:
se_wl_ee = se_fallback_sd/sqrt(n) (default sd=10) for rows missing
se_wl_ee but with a known n, rescuing them from the unusable-row filter.
Unlike placebo_clamp (a one-off per-run judgment call), this is judged
common enough to offer as a standing field: the exact 10/sqrt(n) formula
is documented in redefine1's own curator_note and actually applied (not
just written down) in brenipatide_gzmu_misc5.R and brenipatide_gzmu_gzmd.R
-- three independent sightings of the same convention. Added fixture
Case 9 (a row with se_wl_ee=NA, n known) and verified: regression
(field absent) still drops the row; se_fallback:true rescues it with
the exact expected value (10/sqrt(64)=1.25); missing-reason guard fires.
</commit_message>
<xml_diff>
--- a/.claude/skills/bnma/tests/fixtures/prd_fixture.xlsx
+++ b/.claude/skills/bnma/tests/fixtures/prd_fixture.xlsx
@@ -377,7 +377,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W28"/>
+  <dimension ref="A1:W30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -2575,6 +2575,156 @@
         </is>
       </c>
       <c r="S28" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>20260814</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>se-fallback-1</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>placebo</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>placebo</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>lilly</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>phase 3</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>36 week</t>
+        </is>
+      </c>
+      <c r="I29">
+        <v>64</v>
+      </c>
+      <c r="J29">
+        <v>100</v>
+      </c>
+      <c r="K29">
+        <v>0</v>
+      </c>
+      <c r="L29">
+        <v>1</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>synthetic fixture</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>obese non-t2d</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>mmrm on treatment</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>20260814</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>se-fallback-1</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>hdm2000 5mg qw</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>hdm2000</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>lilly</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>injectable</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>phase 3</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>36 week</t>
+        </is>
+      </c>
+      <c r="I30">
+        <v>64</v>
+      </c>
+      <c r="J30">
+        <v>100</v>
+      </c>
+      <c r="K30">
+        <v>-10</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>publication</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>synthetic fixture</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>obese non-t2d</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>mmrm on treatment</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
         <is>
           <t>fixture</t>
         </is>

</xml_diff>